<commit_message>
Update Backup Checker: fix frozen-exe crash, add GUI
- Fix isatty crash on frozen/windowed builds (sys.stdout is None) that
  broke the desktop GUI on startup.
- Add backup_checker_gui.py (Tkinter desktop front end) and its
  PyInstaller BackupChecker.spec.
- Add a folder-local .gitignore excluding the built exe and generated
  report files.
- Remove stale one-off test report output that had been committed
  previously.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/python/aws/Backups/Backup_Checker/backup_config.xlsx
+++ b/python/aws/Backups/Backup_Checker/backup_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1Aa_uz7RW_XGIeCbQ6gh3B4AQvmMMMBsO\Google - Phenome - IT\HowTos\Itay\Scripts\Backup_Checker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3727F453-6201-4855-9904-E6FC169EDA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7066A14A-BC35-4ACD-8251-309B91A98CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backup Config" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="114">
   <si>
     <t>Phenome Networks — RDS Backup S3 Configuration</t>
   </si>
@@ -376,6 +376,9 @@
   </si>
   <si>
     <t xml:space="preserve">enza-test-database-backup </t>
+  </si>
+  <si>
+    <t>phenome-farm-hannong-mysql-backup</t>
   </si>
 </sst>
 </file>
@@ -469,13 +472,6 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <color rgb="FF0F141A"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="8"/>
       <color rgb="FF656871"/>
       <name val="Arial"/>
@@ -486,6 +482,14 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -545,8 +549,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -601,17 +606,20 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -913,28 +921,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G40"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="49.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="56.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="49.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="56.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:7" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-    </row>
-    <row r="2" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+    </row>
+    <row r="2" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -957,7 +965,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -981,7 +989,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -1005,7 +1013,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -1029,7 +1037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -1053,7 +1061,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -1063,10 +1071,10 @@
       <c r="C7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="E7" s="18" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="4" t="str">
@@ -1077,7 +1085,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -1101,7 +1109,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1125,7 +1133,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -1149,7 +1157,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -1173,7 +1181,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -1197,7 +1205,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -1221,7 +1229,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -1231,17 +1239,21 @@
       <c r="C14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="D14" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>11</v>
+      </c>
       <c r="F14" s="7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>s3://phenome-farm-hannong-mysql-backup/rds_weekly_backup/</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -1265,7 +1277,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -1289,7 +1301,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>15</v>
       </c>
@@ -1313,7 +1325,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -1337,7 +1349,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -1357,7 +1369,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>18</v>
       </c>
@@ -1381,7 +1393,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -1405,7 +1417,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>20</v>
       </c>
@@ -1429,7 +1441,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -1453,7 +1465,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>22</v>
       </c>
@@ -1477,7 +1489,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -1501,7 +1513,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>24</v>
       </c>
@@ -1525,7 +1537,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -1549,7 +1561,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>26</v>
       </c>
@@ -1573,7 +1585,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -1597,7 +1609,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>28</v>
       </c>
@@ -1621,7 +1633,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>29</v>
       </c>
@@ -1645,7 +1657,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>30</v>
       </c>
@@ -1669,7 +1681,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -1689,7 +1701,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>32</v>
       </c>
@@ -1709,7 +1721,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -1729,7 +1741,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>34</v>
       </c>
@@ -1749,7 +1761,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -1769,7 +1781,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>36</v>
       </c>
@@ -1782,7 +1794,7 @@
       <c r="D38" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E38" s="22" t="s">
+      <c r="E38" s="19" t="s">
         <v>11</v>
       </c>
       <c r="F38" s="7" t="str">
@@ -1793,7 +1805,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -1817,7 +1829,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>38</v>
       </c>
@@ -1851,6 +1863,9 @@
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E14" r:id="rId1" display="https://524574648815-6n2hmjzt.ap-northeast-2.console.aws.amazon.com/s3/buckets/phenome-farm-hannong-mysql-backup?prefix=rds_weekly_backup/" xr:uid="{254AA6FF-388F-4B82-A0ED-C998DFDAB461}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1858,124 +1873,124 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="10.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9"/>
     </row>
-    <row r="3" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="10.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
     </row>
-    <row r="11" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" ht="10.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9"/>
     </row>
-    <row r="15" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" ht="10.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9"/>
     </row>
-    <row r="21" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>84</v>
       </c>

</xml_diff>